<commit_message>
Update lotto data (2026-07-04 14:08)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48268,25 +48268,25 @@
       <c r="A1231" s="31" t="n">
         <v>1230</v>
       </c>
-      <c r="B1231" t="n">
+      <c r="B1231" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="C1231" t="n">
+      <c r="C1231" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="D1231" t="n">
+      <c r="D1231" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="E1231" t="n">
+      <c r="E1231" s="27" t="n">
         <v>22</v>
       </c>
-      <c r="F1231" t="n">
+      <c r="F1231" s="27" t="n">
         <v>28</v>
       </c>
-      <c r="G1231" t="n">
+      <c r="G1231" s="27" t="n">
         <v>42</v>
       </c>
-      <c r="H1231" t="n">
+      <c r="H1231" s="27" t="n">
         <v>45</v>
       </c>
       <c r="J1231" s="27">
@@ -48303,7 +48303,30 @@
       </c>
     </row>
     <row r="1232" ht="13.8" customHeight="1" s="28">
-      <c r="A1232" s="31" t="n"/>
+      <c r="A1232" s="31" t="n">
+        <v>1231</v>
+      </c>
+      <c r="B1232" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1232" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1232" t="n">
+        <v>14</v>
+      </c>
+      <c r="E1232" t="n">
+        <v>18</v>
+      </c>
+      <c r="F1232" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1232" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1232" t="n">
+        <v>15</v>
+      </c>
       <c r="J1232" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1232:G1232, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-07-11 14:00)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48306,25 +48306,25 @@
       <c r="A1232" s="31" t="n">
         <v>1231</v>
       </c>
-      <c r="B1232" t="n">
+      <c r="B1232" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="C1232" t="n">
+      <c r="C1232" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1232" t="n">
+      <c r="D1232" s="27" t="n">
         <v>14</v>
       </c>
-      <c r="E1232" t="n">
+      <c r="E1232" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="F1232" t="n">
+      <c r="F1232" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="G1232" t="n">
+      <c r="G1232" s="27" t="n">
         <v>38</v>
       </c>
-      <c r="H1232" t="n">
+      <c r="H1232" s="27" t="n">
         <v>15</v>
       </c>
       <c r="J1232" s="27">
@@ -48341,7 +48341,30 @@
       </c>
     </row>
     <row r="1233" ht="13.8" customHeight="1" s="28">
-      <c r="A1233" s="31" t="n"/>
+      <c r="A1233" s="31" t="n">
+        <v>1232</v>
+      </c>
+      <c r="B1233" t="n">
+        <v>12</v>
+      </c>
+      <c r="C1233" t="n">
+        <v>15</v>
+      </c>
+      <c r="D1233" t="n">
+        <v>19</v>
+      </c>
+      <c r="E1233" t="n">
+        <v>22</v>
+      </c>
+      <c r="F1233" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1233" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1233" t="n">
+        <v>3</v>
+      </c>
       <c r="J1233" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1233:G1233, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-07-18 13:55)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48344,25 +48344,25 @@
       <c r="A1233" s="31" t="n">
         <v>1232</v>
       </c>
-      <c r="B1233" t="n">
+      <c r="B1233" s="27" t="n">
         <v>12</v>
       </c>
-      <c r="C1233" t="n">
+      <c r="C1233" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="D1233" t="n">
+      <c r="D1233" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="E1233" t="n">
+      <c r="E1233" s="27" t="n">
         <v>22</v>
       </c>
-      <c r="F1233" t="n">
+      <c r="F1233" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="G1233" t="n">
+      <c r="G1233" s="27" t="n">
         <v>36</v>
       </c>
-      <c r="H1233" t="n">
+      <c r="H1233" s="27" t="n">
         <v>3</v>
       </c>
       <c r="J1233" s="27">
@@ -48379,7 +48379,30 @@
       </c>
     </row>
     <row r="1234" ht="13.8" customHeight="1" s="28">
-      <c r="A1234" s="31" t="n"/>
+      <c r="A1234" s="31" t="n">
+        <v>1233</v>
+      </c>
+      <c r="B1234" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1234" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1234" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1234" t="n">
+        <v>25</v>
+      </c>
+      <c r="F1234" t="n">
+        <v>37</v>
+      </c>
+      <c r="G1234" t="n">
+        <v>40</v>
+      </c>
+      <c r="H1234" t="n">
+        <v>29</v>
+      </c>
       <c r="J1234" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1234:G1234, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-07-25 14:08)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48382,25 +48382,25 @@
       <c r="A1234" s="31" t="n">
         <v>1233</v>
       </c>
-      <c r="B1234" t="n">
+      <c r="B1234" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="C1234" t="n">
+      <c r="C1234" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="D1234" t="n">
+      <c r="D1234" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E1234" t="n">
+      <c r="E1234" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="F1234" t="n">
+      <c r="F1234" s="27" t="n">
         <v>37</v>
       </c>
-      <c r="G1234" t="n">
+      <c r="G1234" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="H1234" t="n">
+      <c r="H1234" s="27" t="n">
         <v>29</v>
       </c>
       <c r="J1234" s="27">
@@ -48417,7 +48417,30 @@
       </c>
     </row>
     <row r="1235" ht="13.8" customHeight="1" s="28">
-      <c r="A1235" s="31" t="n"/>
+      <c r="A1235" s="31" t="n">
+        <v>1234</v>
+      </c>
+      <c r="B1235" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1235" t="n">
+        <v>15</v>
+      </c>
+      <c r="D1235" t="n">
+        <v>19</v>
+      </c>
+      <c r="E1235" t="n">
+        <v>31</v>
+      </c>
+      <c r="F1235" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1235" t="n">
+        <v>43</v>
+      </c>
+      <c r="H1235" t="n">
+        <v>27</v>
+      </c>
       <c r="J1235" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1235:G1235, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-08-01 14:06)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48420,25 +48420,25 @@
       <c r="A1235" s="31" t="n">
         <v>1234</v>
       </c>
-      <c r="B1235" t="n">
+      <c r="B1235" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="C1235" t="n">
+      <c r="C1235" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="D1235" t="n">
+      <c r="D1235" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="E1235" t="n">
+      <c r="E1235" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="F1235" t="n">
+      <c r="F1235" s="27" t="n">
         <v>35</v>
       </c>
-      <c r="G1235" t="n">
+      <c r="G1235" s="27" t="n">
         <v>43</v>
       </c>
-      <c r="H1235" t="n">
+      <c r="H1235" s="27" t="n">
         <v>27</v>
       </c>
       <c r="J1235" s="27">
@@ -48455,7 +48455,30 @@
       </c>
     </row>
     <row r="1236" ht="13.8" customHeight="1" s="28">
-      <c r="A1236" s="31" t="n"/>
+      <c r="A1236" s="31" t="n">
+        <v>1235</v>
+      </c>
+      <c r="B1236" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1236" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1236" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1236" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1236" t="n">
+        <v>39</v>
+      </c>
+      <c r="G1236" t="n">
+        <v>43</v>
+      </c>
+      <c r="H1236" t="n">
+        <v>20</v>
+      </c>
       <c r="J1236" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1236:G1236, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-08-08 13:26)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48458,25 +48458,25 @@
       <c r="A1236" s="31" t="n">
         <v>1235</v>
       </c>
-      <c r="B1236" t="n">
+      <c r="B1236" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="C1236" t="n">
+      <c r="C1236" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="D1236" t="n">
+      <c r="D1236" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="E1236" t="n">
+      <c r="E1236" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="F1236" t="n">
+      <c r="F1236" s="27" t="n">
         <v>39</v>
       </c>
-      <c r="G1236" t="n">
+      <c r="G1236" s="27" t="n">
         <v>43</v>
       </c>
-      <c r="H1236" t="n">
+      <c r="H1236" s="27" t="n">
         <v>20</v>
       </c>
       <c r="J1236" s="27">
@@ -48493,7 +48493,30 @@
       </c>
     </row>
     <row r="1237" ht="13.8" customHeight="1" s="28">
-      <c r="A1237" s="31" t="n"/>
+      <c r="A1237" s="31" t="n">
+        <v>1236</v>
+      </c>
+      <c r="B1237" t="n">
+        <v>12</v>
+      </c>
+      <c r="C1237" t="n">
+        <v>18</v>
+      </c>
+      <c r="D1237" t="n">
+        <v>21</v>
+      </c>
+      <c r="E1237" t="n">
+        <v>29</v>
+      </c>
+      <c r="F1237" t="n">
+        <v>34</v>
+      </c>
+      <c r="G1237" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1237" t="n">
+        <v>10</v>
+      </c>
       <c r="J1237" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1237:G1237, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-08-15 13:07)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48496,25 +48496,25 @@
       <c r="A1237" s="31" t="n">
         <v>1236</v>
       </c>
-      <c r="B1237" t="n">
+      <c r="B1237" s="27" t="n">
         <v>12</v>
       </c>
-      <c r="C1237" t="n">
+      <c r="C1237" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="D1237" t="n">
+      <c r="D1237" s="27" t="n">
         <v>21</v>
       </c>
-      <c r="E1237" t="n">
+      <c r="E1237" s="27" t="n">
         <v>29</v>
       </c>
-      <c r="F1237" t="n">
+      <c r="F1237" s="27" t="n">
         <v>34</v>
       </c>
-      <c r="G1237" t="n">
+      <c r="G1237" s="27" t="n">
         <v>38</v>
       </c>
-      <c r="H1237" t="n">
+      <c r="H1237" s="27" t="n">
         <v>10</v>
       </c>
       <c r="J1237" s="27">
@@ -48531,7 +48531,30 @@
       </c>
     </row>
     <row r="1238" ht="13.8" customHeight="1" s="28">
-      <c r="A1238" s="31" t="n"/>
+      <c r="A1238" s="31" t="n">
+        <v>1237</v>
+      </c>
+      <c r="B1238" t="n">
+        <v>10</v>
+      </c>
+      <c r="C1238" t="n">
+        <v>20</v>
+      </c>
+      <c r="D1238" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1238" t="n">
+        <v>34</v>
+      </c>
+      <c r="F1238" t="n">
+        <v>37</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>40</v>
+      </c>
+      <c r="H1238" t="n">
+        <v>36</v>
+      </c>
       <c r="J1238" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1238:G1238, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-08-22 13:08)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48534,25 +48534,25 @@
       <c r="A1238" s="31" t="n">
         <v>1237</v>
       </c>
-      <c r="B1238" t="n">
+      <c r="B1238" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="C1238" t="n">
+      <c r="C1238" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="D1238" t="n">
+      <c r="D1238" s="27" t="n">
         <v>23</v>
       </c>
-      <c r="E1238" t="n">
+      <c r="E1238" s="27" t="n">
         <v>34</v>
       </c>
-      <c r="F1238" t="n">
+      <c r="F1238" s="27" t="n">
         <v>37</v>
       </c>
-      <c r="G1238" t="n">
+      <c r="G1238" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="H1238" t="n">
+      <c r="H1238" s="27" t="n">
         <v>36</v>
       </c>
       <c r="J1238" s="27">
@@ -48569,7 +48569,30 @@
       </c>
     </row>
     <row r="1239" ht="13.8" customHeight="1" s="28">
-      <c r="A1239" s="31" t="n"/>
+      <c r="A1239" s="31" t="n">
+        <v>1238</v>
+      </c>
+      <c r="B1239" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1239" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1239" t="n">
+        <v>18</v>
+      </c>
+      <c r="E1239" t="n">
+        <v>32</v>
+      </c>
+      <c r="F1239" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1239" t="n">
+        <v>22</v>
+      </c>
       <c r="J1239" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1239:G1239, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-08-29 16:49)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48572,25 +48572,25 @@
       <c r="A1239" s="31" t="n">
         <v>1238</v>
       </c>
-      <c r="B1239" t="n">
+      <c r="B1239" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="C1239" t="n">
+      <c r="C1239" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1239" t="n">
+      <c r="D1239" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="E1239" t="n">
+      <c r="E1239" s="27" t="n">
         <v>32</v>
       </c>
-      <c r="F1239" t="n">
+      <c r="F1239" s="27" t="n">
         <v>38</v>
       </c>
-      <c r="G1239" t="n">
+      <c r="G1239" s="27" t="n">
         <v>42</v>
       </c>
-      <c r="H1239" t="n">
+      <c r="H1239" s="27" t="n">
         <v>22</v>
       </c>
       <c r="J1239" s="27">
@@ -48607,7 +48607,30 @@
       </c>
     </row>
     <row r="1240" ht="13.8" customHeight="1" s="28">
-      <c r="A1240" s="31" t="n"/>
+      <c r="A1240" s="31" t="n">
+        <v>1239</v>
+      </c>
+      <c r="B1240" t="n">
+        <v>11</v>
+      </c>
+      <c r="C1240" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1240" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1240" t="n">
+        <v>32</v>
+      </c>
+      <c r="F1240" t="n">
+        <v>33</v>
+      </c>
+      <c r="G1240" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1240" t="n">
+        <v>8</v>
+      </c>
       <c r="J1240" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1240:G1240, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-09-05 15:26)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48610,25 +48610,25 @@
       <c r="A1240" s="31" t="n">
         <v>1239</v>
       </c>
-      <c r="B1240" t="n">
+      <c r="B1240" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="C1240" t="n">
+      <c r="C1240" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1240" t="n">
+      <c r="D1240" s="27" t="n">
         <v>22</v>
       </c>
-      <c r="E1240" t="n">
+      <c r="E1240" s="27" t="n">
         <v>32</v>
       </c>
-      <c r="F1240" t="n">
+      <c r="F1240" s="27" t="n">
         <v>33</v>
       </c>
-      <c r="G1240" t="n">
+      <c r="G1240" s="27" t="n">
         <v>36</v>
       </c>
-      <c r="H1240" t="n">
+      <c r="H1240" s="27" t="n">
         <v>8</v>
       </c>
       <c r="J1240" s="27">
@@ -48645,7 +48645,30 @@
       </c>
     </row>
     <row r="1241" ht="13.8" customHeight="1" s="28">
-      <c r="A1241" s="31" t="n"/>
+      <c r="A1241" s="31" t="n">
+        <v>1240</v>
+      </c>
+      <c r="B1241" t="n">
+        <v>11</v>
+      </c>
+      <c r="C1241" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1241" t="n">
+        <v>19</v>
+      </c>
+      <c r="E1241" t="n">
+        <v>20</v>
+      </c>
+      <c r="F1241" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1241" t="n">
+        <v>44</v>
+      </c>
+      <c r="H1241" t="n">
+        <v>27</v>
+      </c>
       <c r="J1241" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1241:G1241, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-09-19 15:59)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48648,25 +48648,25 @@
       <c r="A1241" s="31" t="n">
         <v>1240</v>
       </c>
-      <c r="B1241" t="n">
+      <c r="B1241" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="C1241" t="n">
+      <c r="C1241" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1241" t="n">
+      <c r="D1241" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="E1241" t="n">
+      <c r="E1241" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="F1241" t="n">
+      <c r="F1241" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="G1241" t="n">
+      <c r="G1241" s="27" t="n">
         <v>44</v>
       </c>
-      <c r="H1241" t="n">
+      <c r="H1241" s="27" t="n">
         <v>27</v>
       </c>
       <c r="J1241" s="27">
@@ -48683,7 +48683,30 @@
       </c>
     </row>
     <row r="1242" ht="13.8" customHeight="1" s="28">
-      <c r="A1242" s="31" t="n"/>
+      <c r="A1242" s="31" t="n">
+        <v>1241</v>
+      </c>
+      <c r="B1242" t="n">
+        <v>7</v>
+      </c>
+      <c r="C1242" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1242" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1242" t="n">
+        <v>23</v>
+      </c>
+      <c r="F1242" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1242" t="n">
+        <v>43</v>
+      </c>
+      <c r="H1242" t="n">
+        <v>9</v>
+      </c>
       <c r="J1242" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1242:G1242, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-09-26 16:34)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48686,25 +48686,25 @@
       <c r="A1242" s="31" t="n">
         <v>1241</v>
       </c>
-      <c r="B1242" t="n">
+      <c r="B1242" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="C1242" t="n">
+      <c r="C1242" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1242" t="n">
+      <c r="D1242" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="E1242" t="n">
+      <c r="E1242" s="27" t="n">
         <v>23</v>
       </c>
-      <c r="F1242" t="n">
+      <c r="F1242" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="G1242" t="n">
+      <c r="G1242" s="27" t="n">
         <v>43</v>
       </c>
-      <c r="H1242" t="n">
+      <c r="H1242" s="27" t="n">
         <v>9</v>
       </c>
       <c r="J1242" s="27">
@@ -48721,7 +48721,30 @@
       </c>
     </row>
     <row r="1243" ht="13.8" customHeight="1" s="28">
-      <c r="A1243" s="31" t="n"/>
+      <c r="A1243" s="31" t="n">
+        <v>1242</v>
+      </c>
+      <c r="B1243" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1243" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1243" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1243" t="n">
+        <v>16</v>
+      </c>
+      <c r="F1243" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1243" t="n">
+        <v>41</v>
+      </c>
+      <c r="H1243" t="n">
+        <v>9</v>
+      </c>
       <c r="J1243" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1243:G1243, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-10-03 16:35)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48724,25 +48724,25 @@
       <c r="A1243" s="31" t="n">
         <v>1242</v>
       </c>
-      <c r="B1243" t="n">
+      <c r="B1243" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="C1243" t="n">
+      <c r="C1243" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="D1243" t="n">
+      <c r="D1243" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="E1243" t="n">
+      <c r="E1243" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="F1243" t="n">
+      <c r="F1243" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="G1243" t="n">
+      <c r="G1243" s="27" t="n">
         <v>41</v>
       </c>
-      <c r="H1243" t="n">
+      <c r="H1243" s="27" t="n">
         <v>9</v>
       </c>
       <c r="J1243" s="27">
@@ -48759,7 +48759,30 @@
       </c>
     </row>
     <row r="1244" ht="13.8" customHeight="1" s="28">
-      <c r="A1244" s="31" t="n"/>
+      <c r="A1244" s="31" t="n">
+        <v>1243</v>
+      </c>
+      <c r="B1244" t="n">
+        <v>9</v>
+      </c>
+      <c r="C1244" t="n">
+        <v>18</v>
+      </c>
+      <c r="D1244" t="n">
+        <v>24</v>
+      </c>
+      <c r="E1244" t="n">
+        <v>38</v>
+      </c>
+      <c r="F1244" t="n">
+        <v>43</v>
+      </c>
+      <c r="G1244" t="n">
+        <v>44</v>
+      </c>
+      <c r="H1244" t="n">
+        <v>35</v>
+      </c>
       <c r="J1244" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1244:G1244, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-10-10 17:25)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48762,25 +48762,25 @@
       <c r="A1244" s="31" t="n">
         <v>1243</v>
       </c>
-      <c r="B1244" t="n">
+      <c r="B1244" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="C1244" t="n">
+      <c r="C1244" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="D1244" t="n">
+      <c r="D1244" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="E1244" t="n">
+      <c r="E1244" s="27" t="n">
         <v>38</v>
       </c>
-      <c r="F1244" t="n">
+      <c r="F1244" s="27" t="n">
         <v>43</v>
       </c>
-      <c r="G1244" t="n">
+      <c r="G1244" s="27" t="n">
         <v>44</v>
       </c>
-      <c r="H1244" t="n">
+      <c r="H1244" s="27" t="n">
         <v>35</v>
       </c>
       <c r="J1244" s="27">
@@ -48797,7 +48797,30 @@
       </c>
     </row>
     <row r="1245" ht="13.8" customHeight="1" s="28">
-      <c r="A1245" s="31" t="n"/>
+      <c r="A1245" s="31" t="n">
+        <v>1244</v>
+      </c>
+      <c r="B1245" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1245" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1245" t="n">
+        <v>18</v>
+      </c>
+      <c r="E1245" t="n">
+        <v>26</v>
+      </c>
+      <c r="F1245" t="n">
+        <v>34</v>
+      </c>
+      <c r="G1245" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1245" t="n">
+        <v>25</v>
+      </c>
       <c r="J1245" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1245:G1245, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-10-17 15:48)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48800,25 +48800,25 @@
       <c r="A1245" s="31" t="n">
         <v>1244</v>
       </c>
-      <c r="B1245" t="n">
+      <c r="B1245" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="C1245" t="n">
+      <c r="C1245" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1245" t="n">
+      <c r="D1245" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="E1245" t="n">
+      <c r="E1245" s="27" t="n">
         <v>26</v>
       </c>
-      <c r="F1245" t="n">
+      <c r="F1245" s="27" t="n">
         <v>34</v>
       </c>
-      <c r="G1245" t="n">
+      <c r="G1245" s="27" t="n">
         <v>38</v>
       </c>
-      <c r="H1245" t="n">
+      <c r="H1245" s="27" t="n">
         <v>25</v>
       </c>
       <c r="J1245" s="27">
@@ -48835,7 +48835,30 @@
       </c>
     </row>
     <row r="1246" ht="13.8" customHeight="1" s="28">
-      <c r="A1246" s="31" t="n"/>
+      <c r="A1246" s="31" t="n">
+        <v>1245</v>
+      </c>
+      <c r="B1246" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1246" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1246" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1246" t="n">
+        <v>28</v>
+      </c>
+      <c r="F1246" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1246" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1246" t="n">
+        <v>12</v>
+      </c>
       <c r="J1246" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1246:G1246, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>